<commit_message>
Seguridad y form contacto
</commit_message>
<xml_diff>
--- a/actividadesPR07.xlsx
+++ b/actividadesPR07.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\ProyectosGaman\Comercio-pagweb\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Proyectos\ecommerce\appE-Commerce\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9690557-FBD7-460F-8890-9AFCE6E52A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B6F9FE-D509-48AD-901B-DA6BB429B941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E2F508A3-0155-48CF-98BD-36E835956C58}"/>
+    <workbookView xWindow="-20610" yWindow="8100" windowWidth="20730" windowHeight="11040" xr2:uid="{E2F508A3-0155-48CF-98BD-36E835956C58}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
   <si>
     <t>PR07-01</t>
   </si>
@@ -474,7 +485,16 @@
     <t>ciberseguridad</t>
   </si>
   <si>
-    <t xml:space="preserve">HECHO </t>
+    <t>Doc</t>
+  </si>
+  <si>
+    <t>Faltantes</t>
+  </si>
+  <si>
+    <t>Completos</t>
+  </si>
+  <si>
+    <t>`</t>
   </si>
 </sst>
 </file>
@@ -497,7 +517,7 @@
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -530,12 +550,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -547,12 +561,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -564,29 +593,52 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -896,724 +948,1072 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{453EEA88-F304-4567-8D80-5ED0DF0FE495}">
-  <dimension ref="A1:G73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <dimension ref="A1:I73"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="42.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="42.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.2">
+    <row r="1" spans="1:9" ht="21">
       <c r="A1" s="2" t="s">
         <v>144</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="G1" t="s">
+      <c r="F1" s="4" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="H1" t="s">
+        <v>150</v>
+      </c>
+      <c r="I1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="G2" s="7"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="H2">
+        <f>COUNTIF(F2:F73,0)</f>
+        <v>56</v>
+      </c>
+      <c r="I2">
+        <f>COUNTIF($F$3:$F$74,1)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="30">
+      <c r="A3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="G3" s="7"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+      <c r="C3" s="6"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="G5" s="10"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
+      <c r="C5" s="6"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="30">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
+      <c r="C6" s="6"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
-      <c r="G7" s="7"/>
-    </row>
-    <row r="8" spans="1:7" ht="28.8">
-      <c r="A8" t="s">
+      <c r="C7" s="6"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="G8" s="7"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
+      <c r="C8" s="6"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="G9" s="7"/>
-    </row>
-    <row r="10" spans="1:7" ht="28.8">
-      <c r="A10" t="s">
+      <c r="C9" s="6"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="G10" s="7"/>
-    </row>
-    <row r="11" spans="1:7" ht="28.8">
-      <c r="A11" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="30">
+      <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="5"/>
-    </row>
-    <row r="12" spans="1:7" ht="28.8">
-      <c r="A12" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="30">
+      <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="6"/>
-      <c r="G12" s="9"/>
-    </row>
-    <row r="13" spans="1:7" ht="28.8">
-      <c r="A13" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="30">
+      <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" spans="1:7" ht="28.8">
-      <c r="A14" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="30">
+      <c r="A14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="6"/>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="6"/>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="6"/>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D17" s="5"/>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="30">
+      <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D18" s="5"/>
-    </row>
-    <row r="19" spans="1:7" ht="28.8">
-      <c r="A19" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="30">
+      <c r="A19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="5"/>
-      <c r="G19" s="7"/>
-    </row>
-    <row r="20" spans="1:7" ht="28.8">
-      <c r="A20" t="s">
+      <c r="C19" s="6"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="30">
+      <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="G20" s="7"/>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
+      <c r="C20" s="6"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="5"/>
-      <c r="G21" s="7"/>
-    </row>
-    <row r="22" spans="1:7" ht="28.8">
-      <c r="A22" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="30">
+      <c r="A22" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D22" s="5"/>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="G23" s="10"/>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" t="s">
+      <c r="C23" s="6"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="4"/>
-      <c r="G24" s="7"/>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" t="s">
+      <c r="C24" s="6"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="G25" s="9"/>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" t="s">
+      <c r="C25" s="6"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="5"/>
-      <c r="E26" s="6"/>
-      <c r="G26" s="9"/>
-    </row>
-    <row r="27" spans="1:7" ht="28.8">
-      <c r="A27" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="30">
+      <c r="A27" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D27" s="5"/>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" t="s">
+      <c r="C27" s="4"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D28" s="5"/>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" t="s">
+      <c r="C28" s="4"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D29" s="5"/>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" t="s">
+      <c r="C29" s="4"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D30" s="5"/>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" t="s">
+      <c r="C30" s="4"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="D31" s="5"/>
-      <c r="G31" s="9"/>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" t="s">
+      <c r="C31" s="4"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="E32" s="6"/>
-      <c r="G32" s="9"/>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33" t="s">
+      <c r="C32" s="6"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D33" s="5"/>
-      <c r="E33" s="6"/>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" t="s">
+      <c r="C33" s="4"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="30">
+      <c r="A34" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="6"/>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35" t="s">
+      <c r="C34" s="6"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="5"/>
-    </row>
-    <row r="36" spans="1:7">
-      <c r="A36" t="s">
+      <c r="C35" s="6"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="5"/>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37" t="s">
+      <c r="C36" s="6"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" t="s">
+      <c r="C37" s="6"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D38" s="5"/>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" t="s">
+      <c r="C38" s="4"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D39" s="5"/>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" t="s">
+      <c r="C39" s="4"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="D40" s="5"/>
-    </row>
-    <row r="41" spans="1:7" ht="28.8">
-      <c r="A41" t="s">
+      <c r="C40" s="4"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="30">
+      <c r="A41" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="5"/>
-    </row>
-    <row r="42" spans="1:7">
-      <c r="A42" t="s">
+      <c r="C41" s="6"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C42" s="4"/>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43" t="s">
+      <c r="C42" s="6"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C43" s="4"/>
-      <c r="G43" s="7"/>
-    </row>
-    <row r="44" spans="1:7">
-      <c r="A44" t="s">
+      <c r="C43" s="6"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C44" s="4"/>
-      <c r="G44" s="7"/>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45" t="s">
+      <c r="C44" s="6"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C45" s="4"/>
-      <c r="G45" s="7"/>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46" t="s">
+      <c r="C45" s="6"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C46" s="4"/>
-    </row>
-    <row r="47" spans="1:7">
-      <c r="A47" t="s">
+      <c r="C46" s="6"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C47" s="4"/>
-      <c r="G47" s="7"/>
-    </row>
-    <row r="48" spans="1:7">
-      <c r="A48" t="s">
+      <c r="C47" s="6"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="C48" s="4"/>
-      <c r="G48" s="7"/>
-    </row>
-    <row r="49" spans="1:7">
-      <c r="A49" t="s">
+      <c r="C48" s="6"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C49" s="4"/>
-      <c r="G49" s="7"/>
-    </row>
-    <row r="50" spans="1:7">
-      <c r="A50" t="s">
+      <c r="C49" s="6"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D50" s="5"/>
-    </row>
-    <row r="51" spans="1:7">
-      <c r="A51" t="s">
+      <c r="C50" s="4"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D51" s="5"/>
-      <c r="G51" s="7"/>
-    </row>
-    <row r="52" spans="1:7">
-      <c r="A52" t="s">
+      <c r="C51" s="4"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D52" s="5"/>
-      <c r="E52" s="6"/>
-    </row>
-    <row r="53" spans="1:7">
-      <c r="A53" t="s">
+      <c r="C52" s="4"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D53" s="5"/>
-      <c r="E53" s="6"/>
-    </row>
-    <row r="54" spans="1:7">
-      <c r="A54" t="s">
+      <c r="C53" s="4"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C54" s="4"/>
-      <c r="D54" s="5"/>
-      <c r="G54" s="7"/>
-    </row>
-    <row r="55" spans="1:7">
-      <c r="A55" t="s">
+      <c r="C54" s="6"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C55" s="4"/>
-      <c r="D55" s="5"/>
-    </row>
-    <row r="56" spans="1:7">
-      <c r="A56" t="s">
+      <c r="C55" s="6"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="D56" s="5"/>
-    </row>
-    <row r="57" spans="1:7" ht="28.8">
-      <c r="A57" t="s">
+      <c r="C56" s="4"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="30">
+      <c r="A57" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="D57" s="5"/>
-    </row>
-    <row r="58" spans="1:7">
-      <c r="A58" t="s">
+      <c r="C57" s="4"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="30">
+      <c r="A58" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D58" s="5"/>
-    </row>
-    <row r="59" spans="1:7">
-      <c r="A59" t="s">
+      <c r="C58" s="4"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D59" s="5"/>
-    </row>
-    <row r="60" spans="1:7">
-      <c r="A60" t="s">
+      <c r="C59" s="4"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C60" s="4"/>
-    </row>
-    <row r="61" spans="1:7">
-      <c r="A61" t="s">
+      <c r="C60" s="6"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C61" s="4"/>
-    </row>
-    <row r="62" spans="1:7">
-      <c r="A62" t="s">
+      <c r="C61" s="6"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D62" s="5"/>
-    </row>
-    <row r="63" spans="1:7">
-      <c r="A63" t="s">
+      <c r="C62" s="4"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="D63" s="5"/>
-    </row>
-    <row r="64" spans="1:7">
-      <c r="A64" t="s">
+      <c r="C63" s="4"/>
+      <c r="D63" s="8"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="30">
+      <c r="A64" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D64" s="5"/>
-    </row>
-    <row r="65" spans="1:7">
-      <c r="A65" t="s">
+      <c r="C64" s="4"/>
+      <c r="D64" s="8"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C65" s="4"/>
-    </row>
-    <row r="66" spans="1:7">
-      <c r="A66" t="s">
+      <c r="C65" s="6"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E66" s="6"/>
-    </row>
-    <row r="67" spans="1:7">
-      <c r="A67" t="s">
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="10"/>
+      <c r="F66" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="30">
+      <c r="A67" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E67" s="6"/>
-    </row>
-    <row r="68" spans="1:7" ht="28.8">
-      <c r="A68" t="s">
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="10"/>
+      <c r="F67" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="30">
+      <c r="A68" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" s="5" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="69" spans="1:7">
-      <c r="A69" t="s">
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="30">
+      <c r="A69" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="E69" s="6"/>
-      <c r="G69" s="7"/>
-    </row>
-    <row r="70" spans="1:7">
-      <c r="A70" t="s">
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" s="5" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" ht="28.8">
-      <c r="A71" t="s">
+      <c r="C70" s="4"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="30">
+      <c r="A71" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" s="5" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" ht="86.4">
-      <c r="A72" t="s">
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="105">
+      <c r="A72" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" s="5" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" ht="28.8">
-      <c r="A73" t="s">
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="30">
+      <c r="A73" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" s="5" t="s">
         <v>142</v>
       </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F73">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>